<commit_message>
catalogue: add mustard Signature pilot
</commit_message>
<xml_diff>
--- a/catalogue/csv/velmaya-products.xlsx
+++ b/catalogue/csv/velmaya-products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S13"/>
+  <dimension ref="A1:S12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -460,40 +460,40 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mustard-jacquard-cotton-kurti-set</v>
+        <v>mustard-jacquard-cotton-kurta-set</v>
       </c>
       <c r="B2" t="str">
-        <v>Mustard Jacquard Cotton Kurti Set</v>
+        <v>Mustard Jacquard Cotton Kurta Set</v>
       </c>
       <c r="C2" t="str">
         <v>kurti-sets</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>signature</v>
       </c>
       <c r="E2" t="str">
-        <v>Description to be finalized.</v>
+        <v>A mustard jacquard cotton kurta set woven with an ivory jacquard motif throughout. The kurta has an open, notch-collar neckline and fabric-covered buttons down the front, finished with elbow-length sleeves and a straight 44-inch length. It is fully lined, with functional side pockets. The set comes with matching straight-cut pants and a jacquard cotton dupatta, edged with a woven border and finished with tassels. Includes: kurta, straight-cut pants, and dupatta. Made in India.</v>
       </c>
       <c r="F2" t="str">
-        <v>Jacquard Cotton</v>
+        <v>Jacquard cotton</v>
       </c>
       <c r="G2" t="str">
-        <v>Care instructions to be finalized.</v>
+        <v>Hand wash cold, separately, or dry clean. Do not bleach. Do not wring — reshape and line dry in shade. Iron on the reverse on a low setting, avoiding the button placket and tassels.</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="I2" t="str">
         <v>XS</v>
       </c>
       <c r="J2" t="str">
-        <v>VEL-KS-001-XS</v>
+        <v>VLM-KS-001-XS</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>2250</v>
       </c>
       <c r="M2" t="str">
         <v>0</v>
@@ -505,7 +505,7 @@
         <v/>
       </c>
       <c r="P2" t="str">
-        <v>Fit notes to be finalized.</v>
+        <v>Relaxed through the body with a straight hem; top length 44 inches. Straight-cut pants with a relaxed leg.</v>
       </c>
       <c r="Q2" t="str">
         <v/>
@@ -514,45 +514,45 @@
         <v/>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>01-front.webp;02-detail_closeup.webp</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>mustard-jacquard-cotton-kurti-set</v>
+        <v>mustard-jacquard-cotton-kurta-set</v>
       </c>
       <c r="B3" t="str">
-        <v>Mustard Jacquard Cotton Kurti Set</v>
+        <v>Mustard Jacquard Cotton Kurta Set</v>
       </c>
       <c r="C3" t="str">
         <v>kurti-sets</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>signature</v>
       </c>
       <c r="E3" t="str">
-        <v>Description to be finalized.</v>
+        <v>A mustard jacquard cotton kurta set woven with an ivory jacquard motif throughout. The kurta has an open, notch-collar neckline and fabric-covered buttons down the front, finished with elbow-length sleeves and a straight 44-inch length. It is fully lined, with functional side pockets. The set comes with matching straight-cut pants and a jacquard cotton dupatta, edged with a woven border and finished with tassels. Includes: kurta, straight-cut pants, and dupatta. Made in India.</v>
       </c>
       <c r="F3" t="str">
-        <v>Jacquard Cotton</v>
+        <v>Jacquard cotton</v>
       </c>
       <c r="G3" t="str">
-        <v>Care instructions to be finalized.</v>
+        <v>Hand wash cold, separately, or dry clean. Do not bleach. Do not wring — reshape and line dry in shade. Iron on the reverse on a low setting, avoiding the button placket and tassels.</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="I3" t="str">
         <v>S</v>
       </c>
       <c r="J3" t="str">
-        <v>VEL-KS-001-S</v>
+        <v>VLM-KS-001-S</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>2250</v>
       </c>
       <c r="M3" t="str">
         <v>0</v>
@@ -564,7 +564,7 @@
         <v/>
       </c>
       <c r="P3" t="str">
-        <v>Fit notes to be finalized.</v>
+        <v>Relaxed through the body with a straight hem; top length 44 inches. Straight-cut pants with a relaxed leg.</v>
       </c>
       <c r="Q3" t="str">
         <v/>
@@ -578,40 +578,40 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>mustard-jacquard-cotton-kurti-set</v>
+        <v>mustard-jacquard-cotton-kurta-set</v>
       </c>
       <c r="B4" t="str">
-        <v>Mustard Jacquard Cotton Kurti Set</v>
+        <v>Mustard Jacquard Cotton Kurta Set</v>
       </c>
       <c r="C4" t="str">
         <v>kurti-sets</v>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>signature</v>
       </c>
       <c r="E4" t="str">
-        <v>Description to be finalized.</v>
+        <v>A mustard jacquard cotton kurta set woven with an ivory jacquard motif throughout. The kurta has an open, notch-collar neckline and fabric-covered buttons down the front, finished with elbow-length sleeves and a straight 44-inch length. It is fully lined, with functional side pockets. The set comes with matching straight-cut pants and a jacquard cotton dupatta, edged with a woven border and finished with tassels. Includes: kurta, straight-cut pants, and dupatta. Made in India.</v>
       </c>
       <c r="F4" t="str">
-        <v>Jacquard Cotton</v>
+        <v>Jacquard cotton</v>
       </c>
       <c r="G4" t="str">
-        <v>Care instructions to be finalized.</v>
+        <v>Hand wash cold, separately, or dry clean. Do not bleach. Do not wring — reshape and line dry in shade. Iron on the reverse on a low setting, avoiding the button placket and tassels.</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="I4" t="str">
         <v>M</v>
       </c>
       <c r="J4" t="str">
-        <v>VEL-KS-001-M</v>
+        <v>VLM-KS-001-M</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>2250</v>
       </c>
       <c r="M4" t="str">
         <v>0</v>
@@ -623,7 +623,7 @@
         <v/>
       </c>
       <c r="P4" t="str">
-        <v>Fit notes to be finalized.</v>
+        <v>Relaxed through the body with a straight hem; top length 44 inches. Straight-cut pants with a relaxed leg.</v>
       </c>
       <c r="Q4" t="str">
         <v/>
@@ -637,40 +637,40 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>mustard-jacquard-cotton-kurti-set</v>
+        <v>mustard-jacquard-cotton-kurta-set</v>
       </c>
       <c r="B5" t="str">
-        <v>Mustard Jacquard Cotton Kurti Set</v>
+        <v>Mustard Jacquard Cotton Kurta Set</v>
       </c>
       <c r="C5" t="str">
         <v>kurti-sets</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>signature</v>
       </c>
       <c r="E5" t="str">
-        <v>Description to be finalized.</v>
+        <v>A mustard jacquard cotton kurta set woven with an ivory jacquard motif throughout. The kurta has an open, notch-collar neckline and fabric-covered buttons down the front, finished with elbow-length sleeves and a straight 44-inch length. It is fully lined, with functional side pockets. The set comes with matching straight-cut pants and a jacquard cotton dupatta, edged with a woven border and finished with tassels. Includes: kurta, straight-cut pants, and dupatta. Made in India.</v>
       </c>
       <c r="F5" t="str">
-        <v>Jacquard Cotton</v>
+        <v>Jacquard cotton</v>
       </c>
       <c r="G5" t="str">
-        <v>Care instructions to be finalized.</v>
+        <v>Hand wash cold, separately, or dry clean. Do not bleach. Do not wring — reshape and line dry in shade. Iron on the reverse on a low setting, avoiding the button placket and tassels.</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="I5" t="str">
         <v>L</v>
       </c>
       <c r="J5" t="str">
-        <v>VEL-KS-001-L</v>
+        <v>VLM-KS-001-L</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="L5" t="str">
-        <v/>
+        <v>2250</v>
       </c>
       <c r="M5" t="str">
         <v>0</v>
@@ -682,7 +682,7 @@
         <v/>
       </c>
       <c r="P5" t="str">
-        <v>Fit notes to be finalized.</v>
+        <v>Relaxed through the body with a straight hem; top length 44 inches. Straight-cut pants with a relaxed leg.</v>
       </c>
       <c r="Q5" t="str">
         <v/>
@@ -696,40 +696,40 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>mustard-jacquard-cotton-kurti-set</v>
+        <v>mustard-jacquard-cotton-kurta-set</v>
       </c>
       <c r="B6" t="str">
-        <v>Mustard Jacquard Cotton Kurti Set</v>
+        <v>Mustard Jacquard Cotton Kurta Set</v>
       </c>
       <c r="C6" t="str">
         <v>kurti-sets</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>signature</v>
       </c>
       <c r="E6" t="str">
-        <v>Description to be finalized.</v>
+        <v>A mustard jacquard cotton kurta set woven with an ivory jacquard motif throughout. The kurta has an open, notch-collar neckline and fabric-covered buttons down the front, finished with elbow-length sleeves and a straight 44-inch length. It is fully lined, with functional side pockets. The set comes with matching straight-cut pants and a jacquard cotton dupatta, edged with a woven border and finished with tassels. Includes: kurta, straight-cut pants, and dupatta. Made in India.</v>
       </c>
       <c r="F6" t="str">
-        <v>Jacquard Cotton</v>
+        <v>Jacquard cotton</v>
       </c>
       <c r="G6" t="str">
-        <v>Care instructions to be finalized.</v>
+        <v>Hand wash cold, separately, or dry clean. Do not bleach. Do not wring — reshape and line dry in shade. Iron on the reverse on a low setting, avoiding the button placket and tassels.</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="I6" t="str">
-        <v>XL</v>
+        <v>2XL</v>
       </c>
       <c r="J6" t="str">
-        <v>VEL-KS-001-XL</v>
+        <v>VLM-KS-001-2XL</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="L6" t="str">
-        <v/>
+        <v>2250</v>
       </c>
       <c r="M6" t="str">
         <v>0</v>
@@ -741,7 +741,7 @@
         <v/>
       </c>
       <c r="P6" t="str">
-        <v>Fit notes to be finalized.</v>
+        <v>Relaxed through the body with a straight hem; top length 44 inches. Straight-cut pants with a relaxed leg.</v>
       </c>
       <c r="Q6" t="str">
         <v/>
@@ -755,10 +755,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>mustard-jacquard-cotton-kurti-set</v>
+        <v>lilac-floral-heavy-linen-kurti-set</v>
       </c>
       <c r="B7" t="str">
-        <v>Mustard Jacquard Cotton Kurti Set</v>
+        <v>Lilac Floral Heavy Linen Kurti Set</v>
       </c>
       <c r="C7" t="str">
         <v>kurti-sets</v>
@@ -770,7 +770,7 @@
         <v>Description to be finalized.</v>
       </c>
       <c r="F7" t="str">
-        <v>Jacquard Cotton</v>
+        <v>Heavy Linen</v>
       </c>
       <c r="G7" t="str">
         <v>Care instructions to be finalized.</v>
@@ -779,10 +779,10 @@
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>2XL</v>
+        <v>XS</v>
       </c>
       <c r="J7" t="str">
-        <v>VEL-KS-001-2XL</v>
+        <v>VEL-KS-002-XS</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -838,10 +838,10 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>XS</v>
+        <v>S</v>
       </c>
       <c r="J8" t="str">
-        <v>VEL-KS-002-XS</v>
+        <v>VEL-KS-002-S</v>
       </c>
       <c r="K8" t="str">
         <v/>
@@ -897,10 +897,10 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>S</v>
+        <v>M</v>
       </c>
       <c r="J9" t="str">
-        <v>VEL-KS-002-S</v>
+        <v>VEL-KS-002-M</v>
       </c>
       <c r="K9" t="str">
         <v/>
@@ -956,10 +956,10 @@
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>M</v>
+        <v>L</v>
       </c>
       <c r="J10" t="str">
-        <v>VEL-KS-002-M</v>
+        <v>VEL-KS-002-L</v>
       </c>
       <c r="K10" t="str">
         <v/>
@@ -1015,10 +1015,10 @@
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>L</v>
+        <v>XL</v>
       </c>
       <c r="J11" t="str">
-        <v>VEL-KS-002-L</v>
+        <v>VEL-KS-002-XL</v>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -1074,10 +1074,10 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>XL</v>
+        <v>2XL</v>
       </c>
       <c r="J12" t="str">
-        <v>VEL-KS-002-XL</v>
+        <v>VEL-KS-002-2XL</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -1104,71 +1104,12 @@
         <v/>
       </c>
       <c r="S12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>lilac-floral-heavy-linen-kurti-set</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Lilac Floral Heavy Linen Kurti Set</v>
-      </c>
-      <c r="C13" t="str">
-        <v>kurti-sets</v>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
-      <c r="E13" t="str">
-        <v>Description to be finalized.</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Heavy Linen</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Care instructions to be finalized.</v>
-      </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
-      <c r="I13" t="str">
-        <v>2XL</v>
-      </c>
-      <c r="J13" t="str">
-        <v>VEL-KS-002-2XL</v>
-      </c>
-      <c r="K13" t="str">
-        <v/>
-      </c>
-      <c r="L13" t="str">
-        <v/>
-      </c>
-      <c r="M13" t="str">
-        <v>0</v>
-      </c>
-      <c r="N13" t="str">
-        <v>false</v>
-      </c>
-      <c r="O13" t="str">
-        <v/>
-      </c>
-      <c r="P13" t="str">
-        <v>Fit notes to be finalized.</v>
-      </c>
-      <c r="Q13" t="str">
-        <v/>
-      </c>
-      <c r="R13" t="str">
-        <v/>
-      </c>
-      <c r="S13" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
catalogue: publish Signature mustard jacquard cotton kurta set
</commit_message>
<xml_diff>
--- a/catalogue/csv/velmaya-products.xlsx
+++ b/catalogue/csv/velmaya-products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -496,10 +496,10 @@
         <v>2250</v>
       </c>
       <c r="M2" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N2" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="O2" t="str">
         <v/>
@@ -555,10 +555,10 @@
         <v>2250</v>
       </c>
       <c r="M3" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N3" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="O3" t="str">
         <v/>
@@ -614,10 +614,10 @@
         <v>2250</v>
       </c>
       <c r="M4" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N4" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="O4" t="str">
         <v/>
@@ -673,10 +673,10 @@
         <v>2250</v>
       </c>
       <c r="M5" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N5" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -720,10 +720,10 @@
         <v>2499</v>
       </c>
       <c r="I6" t="str">
-        <v>2XL</v>
+        <v>XL</v>
       </c>
       <c r="J6" t="str">
-        <v>VLM-KS-001-2XL</v>
+        <v>VLM-KS-001-XL</v>
       </c>
       <c r="K6" t="str">
         <v>2499</v>
@@ -732,10 +732,10 @@
         <v>2250</v>
       </c>
       <c r="M6" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N6" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="O6" t="str">
         <v/>
@@ -755,52 +755,52 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>lilac-floral-heavy-linen-kurti-set</v>
+        <v>mustard-jacquard-cotton-kurta-set</v>
       </c>
       <c r="B7" t="str">
-        <v>Lilac Floral Heavy Linen Kurti Set</v>
+        <v>Mustard Jacquard Cotton Kurta Set</v>
       </c>
       <c r="C7" t="str">
         <v>kurti-sets</v>
       </c>
       <c r="D7" t="str">
-        <v/>
+        <v>signature</v>
       </c>
       <c r="E7" t="str">
-        <v>Description to be finalized.</v>
+        <v>A mustard jacquard cotton kurta set woven with an ivory jacquard motif throughout. The kurta has an open, notch-collar neckline and fabric-covered buttons down the front, finished with elbow-length sleeves and a straight 44-inch length. It is fully lined, with functional side pockets. The set comes with matching straight-cut pants and a jacquard cotton dupatta, edged with a woven border and finished with tassels. Includes: kurta, straight-cut pants, and dupatta. Made in India.</v>
       </c>
       <c r="F7" t="str">
-        <v>Heavy Linen</v>
+        <v>Jacquard cotton</v>
       </c>
       <c r="G7" t="str">
-        <v>Care instructions to be finalized.</v>
+        <v>Hand wash cold, separately, or dry clean. Do not bleach. Do not wring — reshape and line dry in shade. Iron on the reverse on a low setting, avoiding the button placket and tassels.</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="I7" t="str">
-        <v>XS</v>
+        <v>2XL</v>
       </c>
       <c r="J7" t="str">
-        <v>VEL-KS-002-XS</v>
+        <v>VLM-KS-001-2XL</v>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>2499</v>
       </c>
       <c r="L7" t="str">
-        <v/>
+        <v>2250</v>
       </c>
       <c r="M7" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="O7" t="str">
         <v/>
       </c>
       <c r="P7" t="str">
-        <v>Fit notes to be finalized.</v>
+        <v>Relaxed through the body with a straight hem; top length 44 inches. Straight-cut pants with a relaxed leg.</v>
       </c>
       <c r="Q7" t="str">
         <v/>
@@ -838,10 +838,10 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>S</v>
+        <v>XS</v>
       </c>
       <c r="J8" t="str">
-        <v>VEL-KS-002-S</v>
+        <v>VEL-KS-002-XS</v>
       </c>
       <c r="K8" t="str">
         <v/>
@@ -897,10 +897,10 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="J9" t="str">
-        <v>VEL-KS-002-M</v>
+        <v>VEL-KS-002-S</v>
       </c>
       <c r="K9" t="str">
         <v/>
@@ -956,10 +956,10 @@
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>L</v>
+        <v>M</v>
       </c>
       <c r="J10" t="str">
-        <v>VEL-KS-002-L</v>
+        <v>VEL-KS-002-M</v>
       </c>
       <c r="K10" t="str">
         <v/>
@@ -1015,10 +1015,10 @@
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>XL</v>
+        <v>L</v>
       </c>
       <c r="J11" t="str">
-        <v>VEL-KS-002-XL</v>
+        <v>VEL-KS-002-L</v>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -1074,10 +1074,10 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>2XL</v>
+        <v>XL</v>
       </c>
       <c r="J12" t="str">
-        <v>VEL-KS-002-2XL</v>
+        <v>VEL-KS-002-XL</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -1107,9 +1107,68 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>lilac-floral-heavy-linen-kurti-set</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Lilac Floral Heavy Linen Kurti Set</v>
+      </c>
+      <c r="C13" t="str">
+        <v>kurti-sets</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>Description to be finalized.</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Heavy Linen</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Care instructions to be finalized.</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v>2XL</v>
+      </c>
+      <c r="J13" t="str">
+        <v>VEL-KS-002-2XL</v>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v>0</v>
+      </c>
+      <c r="N13" t="str">
+        <v>false</v>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v>Fit notes to be finalized.</v>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>